<commit_message>
Declarar los montos sin IVA en el formulario, la carpeta, la presentación, la planilla y el paquete de entrega
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JmsTv5NfzGveoXYqHYwuQV
</commit_message>
<xml_diff>
--- a/XANTRAX_Planilla_Cotizaciones.xlsx
+++ b/XANTRAX_Planilla_Cotizaciones.xlsx
@@ -148,7 +148,7 @@
     <t xml:space="preserve">Montos de referencia</t>
   </si>
   <si>
-    <t xml:space="preserve">Salen de la carpeta DDJJ (Paso 3, decisión de declarar $516 M). Falta definir si la DDJJ se declara con o sin IVA.</t>
+    <t xml:space="preserve">Salen de la carpeta DDJJ (Paso 3, decisión de declarar $516 M). La DDJJ se declara sin IVA, igual que esta comparación.</t>
   </si>
   <si>
     <t xml:space="preserve">Cantidades</t>
@@ -634,7 +634,7 @@
     <t xml:space="preserve">Resumen: mejor oferta contra el monto declarado en la DDJJ</t>
   </si>
   <si>
-    <t xml:space="preserve">Referencia: carpeta DDJJ, Paso 3 (Fase I declarada: $516 M; Fase II indicativa: $130 M). Mejor oferta sin IVA, tomada de «Comparativo».</t>
+    <t xml:space="preserve">Referencia: carpeta DDJJ, Paso 3 (Fase I declarada: $516 M sin IVA; Fase II indicativa: $130 M sin IVA). Mejor oferta sin IVA, tomada de «Comparativo».</t>
   </si>
   <si>
     <t xml:space="preserve">Concepto</t>
@@ -730,7 +730,7 @@
     <t xml:space="preserve">Línea L07 incluye tasas y permisos (O-18), que no se piden a proveedores: cargar la estimación interna en «Comparativo».</t>
   </si>
   <si>
-    <t xml:space="preserve">Si la DDJJ se declara con IVA, comparar contra la referencia con IVA: hoy la comparación es sin IVA.</t>
+    <t xml:space="preserve">La DDJJ se declara sin IVA: las referencias y las ofertas se comparan sobre la misma base.</t>
   </si>
 </sst>
 </file>
@@ -1434,7 +1434,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
         <v>16</v>
       </c>

</xml_diff>